<commit_message>
updated how water supply is calculated
</commit_message>
<xml_diff>
--- a/inputs/location_code_crosswalk_CalSim.xlsx
+++ b/inputs/location_code_crosswalk_CalSim.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/fnufferrodriguez_usbr_gov/Documents/Desktop/eis-appendix-generation/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{9BE2C0AE-041C-44F6-87C0-BC10225BA465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65FD36E7-F64C-4C54-913F-39C68A09D1D8}"/>
+  <xr:revisionPtr revIDLastSave="75" documentId="13_ncr:1_{9BE2C0AE-041C-44F6-87C0-BC10225BA465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FEAA1EA-2EEE-4EF6-B9E6-9E6E55C16807}"/>
   <bookViews>
-    <workbookView xWindow="-33075" yWindow="840" windowWidth="27015" windowHeight="19365" xr2:uid="{14B88182-57F4-4B3C-8644-9F1A6EE53B53}"/>
+    <workbookView xWindow="-76920" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{14B88182-57F4-4B3C-8644-9F1A6EE53B53}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2233" uniqueCount="561">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2260" uniqueCount="571">
   <si>
     <t>QueryID</t>
   </si>
@@ -1719,13 +1719,43 @@
   </si>
   <si>
     <t>D_SAC162_09_SA2</t>
+  </si>
+  <si>
+    <t>DEL_CVP_PSC_N</t>
+  </si>
+  <si>
+    <t>DEL_CVP_PRF_N</t>
+  </si>
+  <si>
+    <t>DEL_CVP_PMI_N_WAMER</t>
+  </si>
+  <si>
+    <t>DEL_CVP_PAG_N</t>
+  </si>
+  <si>
+    <t>SWP_FRSA</t>
+  </si>
+  <si>
+    <t>DEL_CVP_PEX_S</t>
+  </si>
+  <si>
+    <t>DEL_CVP_PRF_S</t>
+  </si>
+  <si>
+    <t>DEL_CVP_PMI_S</t>
+  </si>
+  <si>
+    <t>DEL_CVP_PAG_S</t>
+  </si>
+  <si>
+    <t>DELIVERY-CVP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1791,8 +1821,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1841,8 +1877,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA9D08E"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1881,13 +1923,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1999,6 +2052,11 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2344,10 +2402,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -2646,7 +2700,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0E97D62-E007-4D94-B471-28936CBA853B}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P345"/>
+  <dimension ref="A1:P354"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="2" max="2" width="26.41796875" customWidth="1"/>
@@ -10747,6 +10801,105 @@
         <v>86</v>
       </c>
       <c r="K345" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="346" spans="3:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="I346" s="41" t="s">
+        <v>561</v>
+      </c>
+      <c r="J346" s="43" t="s">
+        <v>570</v>
+      </c>
+      <c r="K346" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="347" spans="3:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="I347" s="42" t="s">
+        <v>562</v>
+      </c>
+      <c r="J347" s="43" t="s">
+        <v>570</v>
+      </c>
+      <c r="K347" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="348" spans="3:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="I348" s="42" t="s">
+        <v>563</v>
+      </c>
+      <c r="J348" s="43" t="s">
+        <v>570</v>
+      </c>
+      <c r="K348" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="349" spans="3:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="I349" s="42" t="s">
+        <v>564</v>
+      </c>
+      <c r="J349" s="43" t="s">
+        <v>570</v>
+      </c>
+      <c r="K349" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="350" spans="3:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="I350" s="42" t="s">
+        <v>565</v>
+      </c>
+      <c r="J350" s="43" t="s">
+        <v>549</v>
+      </c>
+      <c r="K350" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="351" spans="3:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="I351" s="42" t="s">
+        <v>566</v>
+      </c>
+      <c r="J351" s="43" t="s">
+        <v>570</v>
+      </c>
+      <c r="K351" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="352" spans="3:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="I352" s="42" t="s">
+        <v>567</v>
+      </c>
+      <c r="J352" s="43" t="s">
+        <v>570</v>
+      </c>
+      <c r="K352" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="353" spans="9:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="I353" s="42" t="s">
+        <v>568</v>
+      </c>
+      <c r="J353" s="43" t="s">
+        <v>570</v>
+      </c>
+      <c r="K353" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="354" spans="9:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="I354" s="42" t="s">
+        <v>569</v>
+      </c>
+      <c r="J354" s="43" t="s">
+        <v>570</v>
+      </c>
+      <c r="K354" s="11" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>